<commit_message>
Thai BIM 0.7.1: whole-project audit and verified Family10 legacy layers
</commit_message>
<xml_diff>
--- a/examples/extensions/thai_bim/examples/layer-rebar-BBS.xlsx
+++ b/examples/extensions/thai_bim/examples/layer-rebar-BBS.xlsx
@@ -198,7 +198,7 @@
       </c>
       <c r="N2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="O2" s="0" t="inlineStr">
@@ -274,7 +274,7 @@
       </c>
       <c r="N3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="O3" s="0" t="inlineStr">
@@ -360,12 +360,12 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9eff1b0d75184c21</t>
+          <t xml:space="preserve">91768705c3b94b58</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -403,12 +403,12 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ce28abff33d6447e</t>
+          <t xml:space="preserve">28ec3e0daf064dd2</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -446,12 +446,12 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9b2fe769704f4ee9</t>
+          <t xml:space="preserve">90bdc4ef5a2d4bd9</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -489,12 +489,12 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">4c44adf57e974ce1</t>
+          <t xml:space="preserve">f17ecb90061143a9</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -532,12 +532,12 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">3b02303c96f64085</t>
+          <t xml:space="preserve">cad3f5f06e464d32</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -575,12 +575,12 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c0f1ae86807e42da</t>
+          <t xml:space="preserve">90c13e5b6f564661</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -618,12 +618,12 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c83ce6234c7344ff</t>
+          <t xml:space="preserve">6811dd6e2c984671</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -661,12 +661,12 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5d255304afc34cfe</t>
+          <t xml:space="preserve">77c6f05742e44cd7</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -704,12 +704,12 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b5c4d109d29147c1</t>
+          <t xml:space="preserve">f265ec0fcc7c42a3</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -747,12 +747,12 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e9fe8903756d412e</t>
+          <t xml:space="preserve">663669f75eb04c16</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -790,12 +790,12 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0f79c235286f43c5</t>
+          <t xml:space="preserve">1b85298ad16a4985</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -833,12 +833,12 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">09413bb75586468d</t>
+          <t xml:space="preserve">de142d054b644ac0</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -876,12 +876,12 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1c31beb2bef84363</t>
+          <t xml:space="preserve">94b97fe60a2a4f5f</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -919,12 +919,12 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6a5e3a21dde84d8c</t>
+          <t xml:space="preserve">7a6095e169564413</t>
         </is>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -962,12 +962,12 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">85ae5977b35d465b</t>
+          <t xml:space="preserve">4ba4efcd736c48df</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -1005,12 +1005,12 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6849e20d70104e57</t>
+          <t xml:space="preserve">8bf120ac65bb4aa4</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -1048,12 +1048,12 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">17d5ad8450694d22</t>
+          <t xml:space="preserve">f6b3e68529a649de</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -1091,12 +1091,12 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">95bac5f8ba6f4fd1</t>
+          <t xml:space="preserve">b50af117816b41da</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -1134,12 +1134,12 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ae2ed3026ef74e2a</t>
+          <t xml:space="preserve">3616d405670845ac</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -1177,12 +1177,12 @@
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ecd5cfed4b044df6</t>
+          <t xml:space="preserve">d1401570b77b4e46</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -1220,12 +1220,12 @@
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">62ae5aaea032455d</t>
+          <t xml:space="preserve">509e3c7a1d844169</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -1263,12 +1263,12 @@
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">769b1b038cee4899</t>
+          <t xml:space="preserve">31896f1cb4d046ed</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -1306,12 +1306,12 @@
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">d6c76fa8eb594bb1</t>
+          <t xml:space="preserve">c0a725adf9ae4fe3</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -1349,12 +1349,12 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">929fcb44fca2455b</t>
+          <t xml:space="preserve">5a4b6ebee60447cb</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -1392,12 +1392,12 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">2373ba026c864e77</t>
+          <t xml:space="preserve">a69a29c6f05549df</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -1435,12 +1435,12 @@
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">200e98babd334ea7</t>
+          <t xml:space="preserve">bf73d97d952e46df</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -1478,12 +1478,12 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c4f13565fd2443e7</t>
+          <t xml:space="preserve">930dc94779824652</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -1521,12 +1521,12 @@
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">6073537118474963</t>
+          <t xml:space="preserve">93a4d0f0e6754881</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -1564,12 +1564,12 @@
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5d1d040f9f7f421d</t>
+          <t xml:space="preserve">39618a4b13af43df</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">97db1706fa7240c6</t>
+          <t xml:space="preserve">1fc9637bc6124952</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">

</xml_diff>